<commit_message>
mtech amd phd alumini data update, CB&KT data update, phd current sort, guest faculty update
</commit_message>
<xml_diff>
--- a/excels/Cep.xlsx
+++ b/excels/Cep.xlsx
@@ -1,41 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NIT\Documents\PA_Catts\Nitw_WB\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACD4E24C-D157-4DDD-A33D-B344723E05E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{922673B2-0EC7-4FA2-8332-EBE376116D57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Seminars" sheetId="1" r:id="rId1"/>
-    <sheet name="Training" sheetId="2" r:id="rId2"/>
-    <sheet name="FacultyDevelopmentPrograms" sheetId="3" r:id="rId3"/>
-    <sheet name="ShortTermTrainingPrograms" sheetId="4" r:id="rId4"/>
+    <sheet name="Conference_Organised" sheetId="5" r:id="rId1"/>
+    <sheet name="Seminars" sheetId="1" r:id="rId2"/>
+    <sheet name="Training" sheetId="2" r:id="rId3"/>
+    <sheet name="FacultyDevelopmentPrograms" sheetId="3" r:id="rId4"/>
+    <sheet name="ShortTermTrainingPrograms" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="144">
   <si>
     <t>S.No</t>
   </si>
   <si>
-    <t>Seminar Topic</t>
-  </si>
-  <si>
     <t>Brief Description</t>
   </si>
   <si>
@@ -75,12 +76,6 @@
     <t>Sponsored by National Rural Infrastructure Development Agency, Ministry of Rural Development, Govt. of India</t>
   </si>
   <si>
-    <t>Panchayat Raj and PWD Engineers</t>
-  </si>
-  <si>
-    <t>New Technology Initiatives in Rural Roads and Use of Marginal Materials</t>
-  </si>
-  <si>
     <t>Planning, Design, Construction of Culverts and Bridges, New Technology Initiatives in Rural Roads and Use of Marginal Materials</t>
   </si>
   <si>
@@ -135,9 +130,6 @@
     <t>Socio-Economic Impacts of Rural Roads</t>
   </si>
   <si>
-    <t>Dr. S. Shankar, Dr. B. Raguram Prof. C.S.R.K. Prasad</t>
-  </si>
-  <si>
     <t>Rural Road Construction Methods</t>
   </si>
   <si>
@@ -160,13 +152,339 @@
   </si>
   <si>
     <t>No.of Participants</t>
+  </si>
+  <si>
+    <t>Trends and Techniques in Transportation (TETRA1997)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Topic</t>
+  </si>
+  <si>
+    <t>SPARC</t>
+  </si>
+  <si>
+    <t>Safe System Perspective for Indian Mixed Traffic Conditions", (SafeInd 2026)</t>
+  </si>
+  <si>
+    <t>9th Conference on Transportation Systems Engineering and Management</t>
+  </si>
+  <si>
+    <t>5th Colloquium on Transportation Systems Engineering and Management (CTSEM)</t>
+  </si>
+  <si>
+    <t>National Conference on “Evaluation of World Class Technical Institutions – Issues &amp; Concerns (EWCTI2018</t>
+  </si>
+  <si>
+    <t>Dr. M.P. Raju, Managing
+Director, LEA Associates South Asia Pvt. Ltd., New Delhi</t>
+  </si>
+  <si>
+    <t>Seminar/Webinar  Topic</t>
+  </si>
+  <si>
+    <t>Dr. T.S. Reddy, Advisor, LEA Associates South Asia Pvt. Ltd., Hyderabad</t>
+  </si>
+  <si>
+    <t>Mr.P.R.K. Murthy, Director (Projects), Metro Project Implementation Unit, Mumbai ,Metropolitan Region Development Authority, Mumbai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Mr. M.P. Naidu, Project Director, L&amp;T
+Metro Rail Ltd., Hyderabad</t>
+  </si>
+  <si>
+    <t>Mr. R.K. Jha, Senior Advisor and Project Director (Corporate Projects), City and
+Industrial Development Corporation, Navi Mumbai</t>
+  </si>
+  <si>
+    <t>Speaker: Mr. D.B. Srinivas, Associate Vice President,
+Transport Planning Department, Delhi Integrated Multimodal Transit System
+Limited, New Delhi</t>
+  </si>
+  <si>
+    <t>Speaker: Mr. M. Kishore Kumar, Director, M/s.
+Aarvee Associates, Hyderabad</t>
+  </si>
+  <si>
+    <t>Mr. K.V. Ganesh Babu, Vice President, Urban Mass Transit Company
+Ltd., Hyderabad</t>
+  </si>
+  <si>
+    <t>Mr. Kailash Chandra Tiwari, Retired Road Safety Expert, Australia</t>
+  </si>
+  <si>
+    <t>Mr. Rajasekhar Rongali,
+Hyderabad</t>
+  </si>
+  <si>
+    <t>Webinar on “Planning for Urban and Regional Transport Systems Insights and Way Forward” as part of Transportation Engineering Industry Expert Talks</t>
+  </si>
+  <si>
+    <t>Webinar on “Road Safety Auditing for Improved Safety on Roads” as part of Transportation Engineering Industry Expert Talks</t>
+  </si>
+  <si>
+    <t>Webinar on “Infrastructure Development Challenges in India - Role of Transportation Engineers and Planners” as part of Transportation Engineering Industry Expert Talks</t>
+  </si>
+  <si>
+    <t>Webinar on “Mass Rapid Transport System - A Case Study of Hyderabad Metro” as part of Transportation Engineering Industry Expert Talks</t>
+  </si>
+  <si>
+    <t>Webinar on "Concept to Development of Large Transportation Projects - A Case Study of Mumbai Trans Harbor Link” as part of Transportation Engineering Industry Expert Talks</t>
+  </si>
+  <si>
+    <t>Webinar on “Socio-economic Cost of Road Accidents in India” as part of Transportation Engineering Industry Expert Talks</t>
+  </si>
+  <si>
+    <t>Webinar on Prevention of Claims and Disputes in Highway Contracts” as part of Transportation Engineering Industry Expert Talks</t>
+  </si>
+  <si>
+    <t>Webinar on “Planning and Design of Green Field Cities – Case Studies of Gujarat International Finance Tec-City and Amaravati” as part of Transportation Engineering Industry Expert Talks</t>
+  </si>
+  <si>
+    <t>Webinar on “Safety Evaluation at School Zone” as part of Transportation Engineering Industry Expert Talks</t>
+  </si>
+  <si>
+    <t>Webinar on “Future of Pavement Condition Surveys using Sub-mm3D Laser Imaging” as part of Transportation Engineering Industry Expert Talks</t>
+  </si>
+  <si>
+    <t>Emerging trends, modern techniques and research developments across transportation engineering</t>
+  </si>
+  <si>
+    <t>Keeps students and professionals current with evolving practices and new technologies</t>
+  </si>
+  <si>
+    <t>Urban and regional transport planning, land use-transport integration, mobility strategies, public transport</t>
+  </si>
+  <si>
+    <t>Helps design sustainable, efficient transport networks and reduce congestion</t>
+  </si>
+  <si>
+    <t>Safety audit stages (design, construction, operation), hazard identification, crash risk assessment</t>
+  </si>
+  <si>
+    <t>Reduces accidents by detecting safety deficiencies early, before and after road opening</t>
+  </si>
+  <si>
+    <t>Funding, land acquisition, delays, policy and planning issues, the professional's role</t>
+  </si>
+  <si>
+    <t>Prepares engineers to deliver infrastructure projects under real-world constraints</t>
+  </si>
+  <si>
+    <t>Metro planning, design, construction, public-private partnership model, operations</t>
+  </si>
+  <si>
+    <t>Shows how large urban transit systems are developed and run, and supports sustainable urban mobility</t>
+  </si>
+  <si>
+    <t>Project conceptualisation, feasibility, design, construction challenges, sea-link engineering</t>
+  </si>
+  <si>
+    <t>Provides insight into the full lifecycle of mega projects and their management</t>
+  </si>
+  <si>
+    <t>Accident statistics, economic losses, human and social impact, cost estimation methods</t>
+  </si>
+  <si>
+    <t>Supports evidence-based safety policy and investment in accident prevention</t>
+  </si>
+  <si>
+    <t>Contract management, risk allocation, claims causes, dispute resolution mechanisms</t>
+  </si>
+  <si>
+    <t>Reduces project delays and cost overruns, and improves contractual practice in highway projects</t>
+  </si>
+  <si>
+    <t>New city master planning, transport and infrastructure integration, smart city features</t>
+  </si>
+  <si>
+    <t>Guides planning of well-organised new cities with integrated mobility and utilities</t>
+  </si>
+  <si>
+    <t>Pedestrian and child safety, traffic calming, speed management, school zone design</t>
+  </si>
+  <si>
+    <t>Protects vulnerable road users and improves safety around schools</t>
+  </si>
+  <si>
+    <t>Automated pavement surveys, 3D laser imaging, crack and distress detection, data analytics</t>
+  </si>
+  <si>
+    <t>Enables accurate, fast pavement monitoring and better maintenance planning</t>
+  </si>
+  <si>
+    <t>Three-day Training Programme on “Design, Construction and Maintenance of Rural Roads under PMGSY” to the PR Engineers of Andhra Pradesh</t>
+  </si>
+  <si>
+    <t>Two Weeks AICTE/ISTE Sponsored STTP on “Issues in Environmental Pollution due to Road Traffic under Mixed Traffic Conditions” to Engineering College Teachers</t>
+  </si>
+  <si>
+    <t>AICTE/ISTE</t>
+  </si>
+  <si>
+    <t>15 Six-day Training Programmes on “Design, Construction and Maintenance of Rural Roads under PMGSY” to the PR Engineers of Andhra Pradesh</t>
+  </si>
+  <si>
+    <t>Three Day Training Programme on “Innovative Technologies for Low Volume Roads” for the Engineers of Panchayat Raj Engineering Department, Government of Telangana,</t>
+  </si>
+  <si>
+    <t>NRRDA, MoRD, GOI</t>
+  </si>
+  <si>
+    <t>Three Day Training programme on "Innovative Technologies for Low Volume
+Roads" for the Engineers of Panchayat Raj Engineering Department</t>
+  </si>
+  <si>
+    <t>Three Day Training programme on "Innovative Technologies for Low Volume Roads" for the Engineers of Panchayat Raj Engineering Department, Government of AP &amp; TS</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> NRRDA, MoRD, GOI</t>
+  </si>
+  <si>
+    <t>Three Day Executive Development Programme on “New and Innovative Technologies for Construction of Low Volume Roads”, for the Engineers of PRED, GoAP</t>
+  </si>
+  <si>
+    <t>Three Day Executive Development Programme on “New and Innovative Technologies for Construction of Low Volume Roads”, for the PRED Engineers of Telangana and Karnataka</t>
+  </si>
+  <si>
+    <t>Three Day Executive Development Programme on “New and Innovative
+Technologies for Construction of Low Volume Roads”, for the PRED Engineers of
+Telangana</t>
+  </si>
+  <si>
+    <t>Three Day Executive Development Programme on “New and Innovative Technologies for Construction of Low Volume Roads”, for the PRED Engineers of Telangana, Tamil Nadu and AP</t>
+  </si>
+  <si>
+    <t>Five Day GIAN Course on “Emerging Methods for Activity-Travel Demand
+Modelling and Simulation”</t>
+  </si>
+  <si>
+    <t>MHRD, GOI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Prof C.S.R.K. Prasad and  Dr. Arpan Mehar </t>
+  </si>
+  <si>
+    <t>Five Day GIAN Course on “Implementation of Advanced Transportation Management Systems (ATMS)”</t>
+  </si>
+  <si>
+    <t>MHRD, GOI through IIT Kharaghpu</t>
+  </si>
+  <si>
+    <t>Five Day GIAN Course on “Decision Tools for Selection and Evaluation of Transportation Projects</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Prof C.S.R.K. Prasad and  Dr.  Venkaiah Chowdary)</t>
+  </si>
+  <si>
+    <t>MHRD, GOI through IIT Kharagpu</t>
+  </si>
+  <si>
+    <t>Five Day GIAN Course on “Transport and the Environment”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Prof C.S.R.K. Prasad and  Dr. S.Shankar)</t>
+  </si>
+  <si>
+    <t>Five Days Training Program on “Road Safety Engineering Measures</t>
+  </si>
+  <si>
+    <t>AITD, New Delhi and MoRTH</t>
+  </si>
+  <si>
+    <t>Five Day GIAN Course on “Sustainable Mobility and Transportation: Innovative Approaches and Solutions”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Prof C.S.R.K. Prasad and  Dr. K.V.R. Ravi Shankar</t>
+  </si>
+  <si>
+    <t>MHRD, GOI through IIT Kharagpur</t>
+  </si>
+  <si>
+    <t>Five Day GIAN Course on “Transportation in a High Tech, Automated and Connected Vehicle World”</t>
+  </si>
+  <si>
+    <t>Five Day FDP on “Global Road Safety Issues and Challenges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Prof C.S.R.K. Prasad and  Dr. KB
+Raghuram</t>
+  </si>
+  <si>
+    <t>TEQIP-III, NIT Warangal,</t>
+  </si>
+  <si>
+    <t>Three Day Executive Development Program on “New Technology Initiatives in Rural Roads and Use of Marginal Materials</t>
+  </si>
+  <si>
+    <t>NRIDA, MoRD, GO</t>
+  </si>
+  <si>
+    <t>NRIDA, MoRD, GOI</t>
+  </si>
+  <si>
+    <t>Three Day Executive Development Program on “Quality Control, Material Testing
+Procedures and Laboratory Practices”</t>
+  </si>
+  <si>
+    <t>Three Day Executive Development Program on “Road Safety and Road Safety Audit for Rural Roads”</t>
+  </si>
+  <si>
+    <t>NRIDA, MoRD, GOI, New Delhi</t>
+  </si>
+  <si>
+    <t>Three Day Executive Development Program on “Construction and Quality Control of Flexible and Rigid Pavements”</t>
+  </si>
+  <si>
+    <t>Three Day Executive Development Program on “Planning, Design and Construction of PMGSY Roads</t>
+  </si>
+  <si>
+    <t>Prof C.S.R.K. Prasad , Dr. Venkaiah Chowdary and Dr. S. Shankar</t>
+  </si>
+  <si>
+    <t>Dr. S. Shankar, Dr. B. Raghuram Prof. C.S.R.K. Prasad</t>
+  </si>
+  <si>
+    <t>Three Day National Transportation Young Researchers Symposium</t>
+  </si>
+  <si>
+    <t>TEQIP - II</t>
+  </si>
+  <si>
+    <t>Five Day National Transportation Young Researchers Symposium</t>
+  </si>
+  <si>
+    <t>TYReS</t>
+  </si>
+  <si>
+    <t>Diamond Jubilee International Alumni Meet and National Conference on “Transforming NIT Warangal as a World Class Technical Institute – Role of Alumni”</t>
+  </si>
+  <si>
+    <t>A five-day executive development programme on Safety Evaluation of Rural Roads to Panchayat Raj and R&amp;B Engineers</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Prof. C.S.R.K. Prasad,Dr. S. Shankar, Dr. Venkaiah Chowdary, Dr. Ravi Shankar </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> TEQIP-III</t>
+  </si>
+  <si>
+    <t>Five Day FDP on “Global Road Safety Issues and Challenges”</t>
+  </si>
+  <si>
+    <t>A five-day Faculty Development Programme focused on understanding global road safety issues, emerging challenges, and effective strategies for reducing road accidents and improving transportation safety. The programme provides participants with knowledge of road safety practices, traffic management, accident prevention, and sustainable transportation approaches.</t>
+  </si>
+  <si>
+    <t>Global road safety trends and challenges; road accident analysis; traffic management and control; road infrastructure and safety; driver behaviour and road-user safety; intelligent transportation systems; vehicle safety technologies; emergency response and post-crash management; sustainable and safe transportation; road safety policies and best practices.</t>
+  </si>
+  <si>
+    <t>Participants will gain a better understanding of global road safety challenges and accident-prevention strategies. They will be able to identify major road safety risks, understand modern traffic and transportation technologies, apply appropriate road safety measures, and contribute to research, teaching, policy development, and awareness programmes related to safer transportation systems.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -186,6 +504,14 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -208,7 +534,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -217,6 +543,13 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -496,199 +829,113 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E21"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C9FDC84-1073-43EC-A1D3-69738206074E}">
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" customWidth="1"/>
-    <col min="2" max="2" width="16.28515625" customWidth="1"/>
-    <col min="3" max="3" width="35" customWidth="1"/>
-    <col min="4" max="4" width="43.7109375" customWidth="1"/>
-    <col min="5" max="5" width="32.5703125" customWidth="1"/>
+    <col min="2" max="2" width="46.5703125" customWidth="1"/>
+    <col min="3" max="3" width="42.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="B2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D2">
+        <v>2014</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D3">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="B4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
+      <c r="B5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D6">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8">
+        <v>2026</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -696,6 +943,333 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.42578125" customWidth="1"/>
+    <col min="2" max="2" width="56" customWidth="1"/>
+    <col min="3" max="4" width="35" customWidth="1"/>
+    <col min="5" max="5" width="43.7109375" customWidth="1"/>
+    <col min="6" max="6" width="32.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2">
+        <v>1997</v>
+      </c>
+      <c r="E2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="2">
+        <v>2020</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="2">
+        <v>2020</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="2">
+        <v>2020</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="2">
+        <v>2020</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="2">
+        <v>2020</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="2">
+        <v>2020</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="2">
+        <v>2020</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="2">
+        <v>2020</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" s="2">
+        <v>2020</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" s="2">
+        <v>2020</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -711,21 +1285,21 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -734,7 +1308,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -743,7 +1317,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -752,7 +1326,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -761,7 +1335,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -770,7 +1344,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -779,7 +1353,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -788,7 +1362,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -797,7 +1371,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -806,7 +1380,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -1074,9 +1648,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="40" customWidth="1"/>
@@ -1085,142 +1659,144 @@
     <col min="5" max="5" width="24.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>37</v>
-      </c>
+    <row r="2" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D2" t="s">
+        <v>142</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="F2" t="s">
+        <v>139</v>
+      </c>
+      <c r="G2">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>37</v>
-      </c>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>37</v>
-      </c>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>37</v>
-      </c>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>37</v>
-      </c>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>37</v>
-      </c>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>37</v>
-      </c>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>37</v>
-      </c>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>37</v>
-      </c>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -1267,32 +1843,37 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="73.140625" customWidth="1"/>
+    <col min="3" max="3" width="57.28515625" customWidth="1"/>
+    <col min="5" max="6" width="9.140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G1" t="s">
         <v>39</v>
-      </c>
-      <c r="C1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F1" t="s">
-        <v>42</v>
-      </c>
-      <c r="G1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1300,19 +1881,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" t="s">
-        <v>14</v>
+        <v>90</v>
       </c>
       <c r="E2">
-        <v>2021</v>
-      </c>
-      <c r="F2" t="s">
-        <v>15</v>
+        <v>2003</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1320,19 +1892,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
+        <v>91</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>92</v>
       </c>
       <c r="E3">
-        <v>2021</v>
-      </c>
-      <c r="F3" t="s">
-        <v>15</v>
+        <v>2003</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1340,19 +1906,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" t="s">
-        <v>14</v>
+        <v>93</v>
       </c>
       <c r="E4">
-        <v>2022</v>
-      </c>
-      <c r="F4" t="s">
-        <v>15</v>
+        <v>2004</v>
+      </c>
+      <c r="G4">
+        <v>546</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1360,39 +1920,33 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" t="s">
-        <v>20</v>
+        <v>94</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>95</v>
       </c>
       <c r="E5">
-        <v>2022</v>
-      </c>
-      <c r="F5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+        <v>2014</v>
+      </c>
+      <c r="G5">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" t="s">
-        <v>22</v>
+      <c r="B6" s="6" t="s">
+        <v>96</v>
       </c>
       <c r="D6" t="s">
-        <v>14</v>
+        <v>95</v>
       </c>
       <c r="E6">
-        <v>2022</v>
-      </c>
-      <c r="F6" t="s">
-        <v>15</v>
+        <v>2015</v>
+      </c>
+      <c r="G6">
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1400,19 +1954,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" t="s">
-        <v>24</v>
+        <v>97</v>
       </c>
       <c r="D7" t="s">
-        <v>14</v>
+        <v>98</v>
       </c>
       <c r="E7">
-        <v>2022</v>
-      </c>
-      <c r="F7" t="s">
-        <v>15</v>
+        <v>2015</v>
+      </c>
+      <c r="G7">
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1420,19 +1971,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" t="s">
-        <v>26</v>
+        <v>99</v>
       </c>
       <c r="D8" t="s">
-        <v>14</v>
+        <v>95</v>
       </c>
       <c r="E8">
-        <v>2022</v>
-      </c>
-      <c r="F8" t="s">
-        <v>15</v>
+        <v>2016</v>
+      </c>
+      <c r="G8">
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1440,39 +1988,33 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" t="s">
-        <v>24</v>
+        <v>100</v>
       </c>
       <c r="D9" t="s">
-        <v>14</v>
+        <v>95</v>
       </c>
       <c r="E9">
-        <v>2022</v>
-      </c>
-      <c r="F9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>2016</v>
+      </c>
+      <c r="G9">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" t="s">
-        <v>24</v>
+      <c r="B10" s="6" t="s">
+        <v>101</v>
       </c>
       <c r="D10" t="s">
-        <v>14</v>
+        <v>95</v>
       </c>
       <c r="E10">
-        <v>2022</v>
-      </c>
-      <c r="F10" t="s">
-        <v>15</v>
+        <v>2016</v>
+      </c>
+      <c r="G10">
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1480,39 +2022,33 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" t="s">
-        <v>30</v>
+        <v>102</v>
       </c>
       <c r="D11" t="s">
-        <v>14</v>
+        <v>95</v>
       </c>
       <c r="E11">
-        <v>2023</v>
-      </c>
-      <c r="F11" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>2016</v>
+      </c>
+      <c r="G11">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
-        <v>31</v>
+      <c r="B12" s="6" t="s">
+        <v>103</v>
       </c>
       <c r="C12" t="s">
-        <v>32</v>
+        <v>105</v>
       </c>
       <c r="D12" t="s">
-        <v>14</v>
+        <v>104</v>
       </c>
       <c r="E12">
-        <v>2025</v>
-      </c>
-      <c r="F12" t="s">
-        <v>15</v>
+        <v>2016</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1520,19 +2056,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>33</v>
+        <v>106</v>
       </c>
       <c r="C13" t="s">
-        <v>13</v>
+        <v>116</v>
       </c>
       <c r="D13" t="s">
-        <v>14</v>
+        <v>107</v>
       </c>
       <c r="E13">
-        <v>2025</v>
-      </c>
-      <c r="F13" t="s">
-        <v>15</v>
+        <v>2017</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1540,19 +2073,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>108</v>
       </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>109</v>
       </c>
       <c r="D14" t="s">
-        <v>14</v>
+        <v>110</v>
       </c>
       <c r="E14">
-        <v>2025</v>
-      </c>
-      <c r="F14" t="s">
-        <v>15</v>
+        <v>2018</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1560,22 +2090,397 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C15" t="s">
+        <v>112</v>
+      </c>
+      <c r="D15" t="s">
+        <v>110</v>
+      </c>
+      <c r="E15">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>113</v>
+      </c>
+      <c r="D16" t="s">
+        <v>114</v>
+      </c>
+      <c r="E16">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>115</v>
+      </c>
+      <c r="C17" t="s">
+        <v>116</v>
+      </c>
+      <c r="D17" t="s">
+        <v>117</v>
+      </c>
+      <c r="E17">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>118</v>
+      </c>
+      <c r="C18" t="s">
+        <v>105</v>
+      </c>
+      <c r="D18" t="s">
+        <v>117</v>
+      </c>
+      <c r="E18">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>119</v>
+      </c>
+      <c r="C19" t="s">
+        <v>120</v>
+      </c>
+      <c r="D19" t="s">
+        <v>121</v>
+      </c>
+      <c r="E19">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>122</v>
+      </c>
+      <c r="D20" t="s">
+        <v>124</v>
+      </c>
+      <c r="E20">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>21</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D21" t="s">
+        <v>123</v>
+      </c>
+      <c r="E21">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>22</v>
+      </c>
+      <c r="B22" t="s">
+        <v>126</v>
+      </c>
+      <c r="D22" t="s">
+        <v>127</v>
+      </c>
+      <c r="E22">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>23</v>
+      </c>
+      <c r="B23" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>128</v>
+      </c>
+      <c r="C24" t="s">
+        <v>130</v>
+      </c>
+      <c r="D24" t="s">
+        <v>127</v>
+      </c>
+      <c r="E24">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>129</v>
+      </c>
+      <c r="C25" t="s">
+        <v>130</v>
+      </c>
+      <c r="D25" t="s">
+        <v>127</v>
+      </c>
+      <c r="E25">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" t="s">
+        <v>13</v>
+      </c>
+      <c r="E26">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" t="s">
+        <v>13</v>
+      </c>
+      <c r="E28">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" t="s">
+        <v>21</v>
+      </c>
+      <c r="D29" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30" t="s">
+        <v>23</v>
+      </c>
+      <c r="D30" t="s">
+        <v>13</v>
+      </c>
+      <c r="E30">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C31" t="s">
+        <v>21</v>
+      </c>
+      <c r="D31" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>25</v>
+      </c>
+      <c r="C32" t="s">
+        <v>21</v>
+      </c>
+      <c r="D32" t="s">
+        <v>13</v>
+      </c>
+      <c r="E32">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>26</v>
+      </c>
+      <c r="C33" t="s">
+        <v>27</v>
+      </c>
+      <c r="D33" t="s">
+        <v>13</v>
+      </c>
+      <c r="E33">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>32</v>
+      </c>
+      <c r="C34" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>137</v>
+      </c>
+      <c r="C35" t="s">
+        <v>138</v>
+      </c>
+      <c r="E35">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>34</v>
+      </c>
+      <c r="B36" t="s">
+        <v>28</v>
+      </c>
+      <c r="C36" t="s">
+        <v>29</v>
+      </c>
+      <c r="D36" t="s">
+        <v>13</v>
+      </c>
+      <c r="E36">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>35</v>
+      </c>
+      <c r="B37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37" t="s">
+        <v>13</v>
+      </c>
+      <c r="E37">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38">
         <v>36</v>
       </c>
-      <c r="C15" t="s">
+      <c r="B38" t="s">
+        <v>31</v>
+      </c>
+      <c r="C38" t="s">
+        <v>131</v>
+      </c>
+      <c r="D38" t="s">
         <v>13</v>
       </c>
-      <c r="D15" t="s">
-        <v>14</v>
-      </c>
-      <c r="E15">
-        <v>2024</v>
-      </c>
-      <c r="F15" t="s">
-        <v>15</v>
-      </c>
-    </row>
+      <c r="E38">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>